<commit_message>
New Updated Excel Sheets
</commit_message>
<xml_diff>
--- a/NB_LEFT_POINTS.xlsx
+++ b/NB_LEFT_POINTS.xlsx
@@ -663,10 +663,8 @@
         </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="200"/>
+        <crossAx val="100"/>
         <lblOffset val="100"/>
-        <tickLblSkip val="1"/>
-        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -693,7 +691,7 @@
         <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="100"/>
+        <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>

</xml_diff>